<commit_message>
Add htn control diabetes subgroup function
</commit_message>
<xml_diff>
--- a/scenarios/scenarios_aim1/aim1_results_tables.xlsx
+++ b/scenarios/scenarios_aim1/aim1_results_tables.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t xml:space="preserve">Table 1. Cumulative deaths averted (2025-2050) by intervention scenario.</t>
   </si>
@@ -29,13 +29,40 @@
     <t xml:space="preserve">Average per year (thousands)</t>
   </si>
   <si>
+    <t xml:space="preserve">61.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,455.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78.41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,136.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,959.9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Improved Hypertension Control</t>
   </si>
   <si>
-    <t xml:space="preserve">71.05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2,842.1</t>
+    <t xml:space="preserve">20.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">827.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improved Statin Uptake</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">850.5</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Deaths averted (millions) by intervention and cause of death.</t>
@@ -56,16 +83,25 @@
     <t xml:space="preserve">Ischemic stroke</t>
   </si>
   <si>
-    <t xml:space="preserve">4.66</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35.96</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17.99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.44</t>
+    <t xml:space="preserve">0.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">–</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20.85</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.46</t>
   </si>
   <si>
     <t xml:space="preserve">Table 3. Deaths averted by age group and intervention.</t>
@@ -92,73 +128,118 @@
     <t xml:space="preserve">&lt;70</t>
   </si>
   <si>
-    <t xml:space="preserve">227,826,554</t>
-  </si>
-  <si>
-    <t xml:space="preserve">247,214,073</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19,387,519</t>
-  </si>
-  <si>
-    <t xml:space="preserve">775,501</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.8%</t>
+    <t xml:space="preserve">167,028,201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">175,228,222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8,200,022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">328,001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">168,914,734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,313,488</t>
+  </si>
+  <si>
+    <t xml:space="preserve">252,540</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.6%</t>
   </si>
   <si>
     <t xml:space="preserve">70-79</t>
   </si>
   <si>
-    <t xml:space="preserve">273,810,907</t>
-  </si>
-  <si>
-    <t xml:space="preserve">291,467,333</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17,656,426</t>
-  </si>
-  <si>
-    <t xml:space="preserve">706,257</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.1%</t>
+    <t xml:space="preserve">176,788,396</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180,543,266</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,754,870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150,195</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">174,222,070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6,321,196</t>
+  </si>
+  <si>
+    <t xml:space="preserve">252,848</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5%</t>
   </si>
   <si>
     <t xml:space="preserve">80-89</t>
   </si>
   <si>
-    <t xml:space="preserve">385,540,942</t>
-  </si>
-  <si>
-    <t xml:space="preserve">413,222,379</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27,681,437</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,107,257</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.7%</t>
+    <t xml:space="preserve">235,085,787</t>
+  </si>
+  <si>
+    <t xml:space="preserve">242,126,243</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,040,455</t>
+  </si>
+  <si>
+    <t xml:space="preserve">281,618</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">235,086,128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7,040,115</t>
+  </si>
+  <si>
+    <t xml:space="preserve">281,605</t>
   </si>
   <si>
     <t xml:space="preserve">90+</t>
   </si>
   <si>
-    <t xml:space="preserve">159,771,898</t>
-  </si>
-  <si>
-    <t xml:space="preserve">166,099,752</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,327,853</t>
-  </si>
-  <si>
-    <t xml:space="preserve">253,114</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.8%</t>
+    <t xml:space="preserve">96,623,090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">98,308,065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,684,975</t>
+  </si>
+  <si>
+    <t xml:space="preserve">67,399</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.7%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">96,719,479</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,588,586</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63,543</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.6%</t>
   </si>
   <si>
     <t xml:space="preserve">Table 4. Country-level deaths averted (All Interventions, 2025-2050).</t>
@@ -542,14 +623,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
+      <c r="A4"/>
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5">
+      <c r="A5"/>
+      <c r="B5" t="s">
         <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6"/>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -572,41 +691,58 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -631,122 +767,214 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="E7" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" t="s">
+        <v>64</v>
+      </c>
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>71</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
+        <v>73</v>
+      </c>
+      <c r="G11" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -771,30 +999,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>